<commit_message>
what are the system requirements part(proposed_design)
</commit_message>
<xml_diff>
--- a/database/databases/standards_database_master.xlsx
+++ b/database/databases/standards_database_master.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_A14784B15D427AD256A17A52A4DDEA4E22C1BCE0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB9BAB3F-5219-4CB7-92EF-283D7F9AFEB3}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="11_A14784B15D427AD256A17A52A4DDEA4E22C1BCE0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BAD422F-A39F-4658-917B-323688FF74B2}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Standards List" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="183">
   <si>
     <r>
       <t>System</t>
@@ -123,37 +123,499 @@
     <t>booster connection </t>
   </si>
   <si>
+    <t>Fire hydrant systems </t>
+  </si>
+  <si>
+    <t>Hydrant valves</t>
+  </si>
+  <si>
+    <t>NCC Part E1 </t>
+  </si>
+  <si>
+    <t>hydrant pipework</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes </t>
+  </si>
+  <si>
+    <t>booster assembly</t>
+  </si>
+  <si>
+    <t>50 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No </t>
+  </si>
+  <si>
+    <t>Fire hose reels </t>
+  </si>
+  <si>
+    <t>Hose reels</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -  </t>
+  </si>
+  <si>
+    <t>cabinets</t>
+  </si>
+  <si>
+    <t> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">pipework </t>
+  </si>
+  <si>
+    <t>Portable fire extinguishers </t>
+  </si>
+  <si>
+    <t>Extinguishers</t>
+  </si>
+  <si>
+    <t>always</t>
+  </si>
+  <si>
+    <t>brackets</t>
+  </si>
+  <si>
+    <t>cabinet</t>
+  </si>
+  <si>
+    <t>weather protection</t>
+  </si>
+  <si>
+    <t>Fire detection systems </t>
+  </si>
+  <si>
+    <t>Smoke detectors</t>
+  </si>
+  <si>
+    <t>NCC Part E2 / Specification 20 </t>
+  </si>
+  <si>
+    <t>Alarm / warning systems </t>
+  </si>
+  <si>
+    <t>Fire indicator panel</t>
+  </si>
+  <si>
+    <t>NCC Part E4 / Specification 20 </t>
+  </si>
+  <si>
+    <t>sounder</t>
+  </si>
+  <si>
+    <t>building class</t>
+  </si>
+  <si>
+    <t>based on NCC/AS 1670.1</t>
+  </si>
+  <si>
+    <t>strobes</t>
+  </si>
+  <si>
+    <t>hearing-imparied occupants</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> speakers </t>
+  </si>
+  <si>
+    <t>building height/ NCC</t>
+  </si>
+  <si>
+    <t>EWIS present</t>
+  </si>
+  <si>
+    <t>EWIS</t>
+  </si>
+  <si>
+    <t>effective height &gt;</t>
+  </si>
+  <si>
+    <t>manual call points</t>
+  </si>
+  <si>
+    <t>fire detection system exits in building</t>
+  </si>
+  <si>
+    <t>cabling </t>
+  </si>
+  <si>
+    <t>Emergency lighting </t>
+  </si>
+  <si>
+    <t>Emergency luminaires</t>
+  </si>
+  <si>
+    <t>NCC Part E4 </t>
+  </si>
+  <si>
+    <t>exit luminaires</t>
+  </si>
+  <si>
+    <t>exit sign installed</t>
+  </si>
+  <si>
+    <t>central battery system</t>
+  </si>
+  <si>
+    <t>battery type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">central battery </t>
+  </si>
+  <si>
+    <t>local battery packs</t>
+  </si>
+  <si>
+    <t>self-contained</t>
+  </si>
+  <si>
+    <t xml:space="preserve">emergency lighting cabling </t>
+  </si>
+  <si>
+    <t>Exit signs / direction signs </t>
+  </si>
+  <si>
+    <t>Exit signs</t>
+  </si>
+  <si>
+    <t>exit required</t>
+  </si>
+  <si>
+    <t>NCC Part E4 / Specification 25 </t>
+  </si>
+  <si>
+    <t>direction signs</t>
+  </si>
+  <si>
+    <t>exit not immediately visible</t>
+  </si>
+  <si>
+    <t>photoluminescent exit signs</t>
+  </si>
+  <si>
+    <t>electrical supply not required</t>
+  </si>
+  <si>
+    <t>mounting brackets/fixings</t>
+  </si>
+  <si>
+    <t>Smoke Hazard management</t>
+  </si>
+  <si>
+    <t>Smoke exhaust fans</t>
+  </si>
+  <si>
+    <t>Floor Area&gt;</t>
+  </si>
+  <si>
+    <t>2000m2</t>
+  </si>
+  <si>
+    <t>NCC part E2 / E2D2</t>
+  </si>
+  <si>
+    <t>Stair Pressurization</t>
+  </si>
+  <si>
+    <t>Effective height&gt;</t>
+  </si>
+  <si>
+    <t>NCC part E2 / AS 1668.1</t>
+  </si>
+  <si>
+    <t>Smoke Dampers</t>
+  </si>
+  <si>
+    <t>Ductwork</t>
+  </si>
+  <si>
+    <t>If duct penetrates through fire proof wall</t>
+  </si>
+  <si>
+    <t>NCC part C / specification 11, NCC part E2</t>
+  </si>
+  <si>
+    <t>Smoke exhaust/stair pressurization</t>
+  </si>
+  <si>
+    <t>NCC Part E2 / Specification 21</t>
+  </si>
+  <si>
+    <t>control cabling</t>
+  </si>
+  <si>
+    <t>Smoke and heat vents</t>
+  </si>
+  <si>
+    <t>roof vents</t>
+  </si>
+  <si>
+    <t>NCC Part E2 / Specification 22</t>
+  </si>
+  <si>
+    <t>NCC Part E2 / Specification 22/ AS 2665</t>
+  </si>
+  <si>
+    <t>Vent actuators</t>
+  </si>
+  <si>
+    <t>automatic vent installed</t>
+  </si>
+  <si>
+    <t>Fire doors / smoke doors</t>
+  </si>
+  <si>
+    <t>Fire doors</t>
+  </si>
+  <si>
+    <t>FRL required</t>
+  </si>
+  <si>
+    <t>NCC part C4 / C4D2</t>
+  </si>
+  <si>
+    <t>Smoke doors</t>
+  </si>
+  <si>
+    <t>Smoke compartments needed</t>
+  </si>
+  <si>
+    <t>NCC part C4 / C4/D3</t>
+  </si>
+  <si>
+    <t>Closers</t>
+  </si>
+  <si>
+    <t>Fire doors/smoke doors used</t>
+  </si>
+  <si>
+    <t>NCC specification 12</t>
+  </si>
+  <si>
+    <t>Seals</t>
+  </si>
+  <si>
+    <t>Smoke doors used</t>
+  </si>
+  <si>
+    <t>NCC S12C4</t>
+  </si>
+  <si>
+    <t>Hold open devices</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Fire shutters/ fire windows</t>
+  </si>
+  <si>
+    <t>Fire shutters </t>
+  </si>
+  <si>
+    <t>fire-rated glazing  </t>
+  </si>
+  <si>
+    <t>fire windows </t>
+  </si>
+  <si>
+    <t>fire-rated glazing installed</t>
+  </si>
+  <si>
+    <t>Fire stopping/penetration seals</t>
+  </si>
+  <si>
+    <t>Fire collars </t>
+  </si>
+  <si>
+    <t>sealants </t>
+  </si>
+  <si>
+    <t>ductwork penetrates through fireproof element</t>
+  </si>
+  <si>
+    <t>fire pillows </t>
+  </si>
+  <si>
+    <t>cable/pipe penetration systems </t>
+  </si>
+  <si>
     <t>Building class</t>
   </si>
   <si>
-    <t>Fire Hydrant</t>
-  </si>
-  <si>
-    <t>Hose Reel</t>
-  </si>
-  <si>
-    <t>Alarm</t>
-  </si>
-  <si>
-    <t>conditional</t>
+    <t>Stair pressurization</t>
+  </si>
+  <si>
+    <t>Smoke dampers</t>
+  </si>
+  <si>
+    <t>Smoke ductwork</t>
+  </si>
+  <si>
+    <t>Door Closers</t>
+  </si>
+  <si>
+    <t>Door seals</t>
+  </si>
+  <si>
+    <t>Sealants</t>
+  </si>
+  <si>
+    <t>2 (Apartments)</t>
+  </si>
+  <si>
+    <t>No - exempt</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D4</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D3</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory for all openings required to have FRL</t>
+  </si>
+  <si>
+    <t>3 (hotels/hostels)</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D5</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D4</t>
+  </si>
+  <si>
+    <t>5 (offices)</t>
+  </si>
+  <si>
+    <t>conditional (if building requires)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditional - Mandatory if effective height &gt;25m AND &gt;18,000 m² floor area or &gt;108,000 m³ volume (E1D10) </t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D6</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D5</t>
+  </si>
+  <si>
+    <t>Conditional - Required only where active exhaust installed.</t>
+  </si>
+  <si>
+    <t>6 (retail)</t>
+  </si>
+  <si>
+    <t>conditional  (if floor area &gt; 3500m2, volume &gt; 21000m3)</t>
+  </si>
+  <si>
+    <t>Conditional - E2D14/E2D15: additional requirements apply to Cl 6 fire compartments &gt;2,000 m².</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D7</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D6</t>
+  </si>
+  <si>
+    <t>7 (carparks/storage)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conditional (if a separated building) </t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D8</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D7</t>
+  </si>
+  <si>
+    <t>8 (electricity network)</t>
+  </si>
+  <si>
+    <t>conditional (if floor area &gt; 200m2)</t>
+  </si>
+  <si>
+    <t>conditional (if can be connected to town main supply)</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D9</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D8</t>
+  </si>
+  <si>
+    <t>9a (healthcare)</t>
+  </si>
+  <si>
+    <t>Conditional - E2D11: smoke detection + HVAC shutdown required if rise in storeys &gt;2, E1D10 applies also</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D10</t>
+  </si>
+  <si>
+    <t>9b (early childhood centre)</t>
+  </si>
+  <si>
+    <t>conditional (if rise in storeys &lt;2)</t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D11</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D10</t>
+  </si>
+  <si>
+    <t>9c (aged care)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditional - (E1D10) </t>
+  </si>
+  <si>
+    <t>Conditional - Mandatory if effective height &gt;25m E2D12</t>
+  </si>
+  <si>
+    <t>Conditional - required whenever HVAC ducts penetrate fire barriers E2D11</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>NCC E1D4</t>
+  </si>
+  <si>
+    <t>NCC E1D2</t>
+  </si>
+  <si>
+    <t>NCC E1D3</t>
+  </si>
+  <si>
+    <t>NCC E1D14</t>
+  </si>
+  <si>
+    <t>NCC S31C15</t>
+  </si>
+  <si>
+    <t>NCC S31C18/ AS1670.1</t>
+  </si>
+  <si>
+    <t>NCC E4V1</t>
+  </si>
+  <si>
+    <t>NCC E4D5/ E4D6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -167,6 +629,46 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -177,12 +679,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF6C5AC"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -231,39 +733,167 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,59 +1210,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
     <col min="3" max="3" width="19.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" customWidth="1"/>
-    <col min="6" max="6" width="33.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="37.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -644,7 +1274,7 @@
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -652,7 +1282,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -664,7 +1294,7 @@
       <c r="D4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
@@ -672,7 +1302,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -692,27 +1322,27 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -724,12 +1354,924 @@
       <c r="D7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="30.75">
+      <c r="A21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="30.75">
+      <c r="A22" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="30.75">
+      <c r="A23" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="29.25" customHeight="1">
+      <c r="A25" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A27" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="18" customHeight="1">
+      <c r="A29" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="17.25" customHeight="1">
+      <c r="A31" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="21" customHeight="1">
+      <c r="A33" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="20.25" customHeight="1">
+      <c r="A34" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="20.25" customHeight="1">
+      <c r="A35" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F35" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C38" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" s="19"/>
+      <c r="F41" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" s="19"/>
+      <c r="F42" s="24" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B46" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E46" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E47" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B49" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B50" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B51" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="19"/>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B52" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B53" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="19"/>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B54" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B55" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D55" s="19"/>
+      <c r="E55" s="19"/>
+      <c r="F55" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -738,87 +2280,467 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E74BA0-7F06-4379-B08B-B53AE5242141}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
     <col min="3" max="3" width="22.140625" customWidth="1"/>
     <col min="4" max="4" width="21.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" customWidth="1"/>
+    <col min="9" max="9" width="23.42578125" customWidth="1"/>
+    <col min="10" max="18" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:18">
+      <c r="A1" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="5" t="str">
-        <f>'Standards List'!A2</f>
-        <v>Sprinkler systems </v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="3">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="D1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" t="s">
+        <v>82</v>
+      </c>
+      <c r="K1" t="s">
+        <v>129</v>
+      </c>
+      <c r="L1" t="s">
+        <v>130</v>
+      </c>
+      <c r="M1" t="s">
+        <v>131</v>
+      </c>
+      <c r="N1" t="s">
+        <v>103</v>
+      </c>
+      <c r="O1" t="s">
+        <v>106</v>
+      </c>
+      <c r="P1" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>133</v>
+      </c>
+      <c r="R1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="A2" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="3">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="3">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
+      <c r="C2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>136</v>
+      </c>
+      <c r="K2" t="s">
+        <v>137</v>
+      </c>
+      <c r="L2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K3" t="s">
+        <v>141</v>
+      </c>
+      <c r="L3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" t="s">
+        <v>145</v>
+      </c>
+      <c r="K4" t="s">
+        <v>146</v>
+      </c>
+      <c r="L4" t="s">
+        <v>147</v>
+      </c>
+      <c r="M4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" t="s">
+        <v>151</v>
+      </c>
+      <c r="K5" t="s">
+        <v>152</v>
+      </c>
+      <c r="L5" t="s">
+        <v>153</v>
+      </c>
+      <c r="M5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" t="s">
+        <v>156</v>
+      </c>
+      <c r="L6" t="s">
+        <v>157</v>
+      </c>
+      <c r="M6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
+      <c r="A7" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s">
+        <v>161</v>
+      </c>
+      <c r="L7" t="s">
+        <v>162</v>
+      </c>
+      <c r="M7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18">
+      <c r="A8" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" t="s">
+        <v>164</v>
+      </c>
+      <c r="K8" t="s">
+        <v>165</v>
+      </c>
+      <c r="L8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18">
+      <c r="A9" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s">
+        <v>168</v>
+      </c>
+      <c r="L9" t="s">
+        <v>169</v>
+      </c>
+      <c r="M9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18">
+      <c r="A10" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" t="s">
+        <v>171</v>
+      </c>
+      <c r="K10" t="s">
+        <v>172</v>
+      </c>
+      <c r="L10" t="s">
+        <v>173</v>
+      </c>
+      <c r="M10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18">
+      <c r="A11" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="I11" s="19" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>